<commit_message>
Fix ChartQAPro answer extraction in benchmark summaries
</commit_message>
<xml_diff>
--- a/results/qwen25vl3b_trace_candidate37_200_results.xlsx
+++ b/results/qwen25vl3b_trace_candidate37_200_results.xlsx
@@ -1942,25 +1942,25 @@
         <v>113</v>
       </c>
       <c r="E7">
-        <v>29.60157458661558</v>
+        <v>30.37836030090129</v>
       </c>
       <c r="F7">
         <v>200</v>
       </c>
       <c r="G7">
-        <v>15.04636223991063</v>
+        <v>25.43709045963145</v>
       </c>
       <c r="H7">
         <v>200</v>
       </c>
       <c r="I7">
-        <v>13.09814611008896</v>
+        <v>26.27834642448045</v>
       </c>
       <c r="J7">
         <v>200</v>
       </c>
       <c r="K7">
-        <v>10.34287564525967</v>
+        <v>24.9061602772943</v>
       </c>
       <c r="L7">
         <v>200</v>
@@ -3152,16 +3152,16 @@
         <v>88</v>
       </c>
       <c r="E39">
-        <v>33.84963332591977</v>
+        <v>33.87062753441398</v>
       </c>
       <c r="G39">
-        <v>34.5020744883892</v>
+        <v>34.78290498081409</v>
       </c>
       <c r="I39">
-        <v>35.76300521084337</v>
+        <v>36.11922684096206</v>
       </c>
       <c r="K39">
-        <v>34.43570976558318</v>
+        <v>34.82931205293546</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -3172,16 +3172,16 @@
         <v>89</v>
       </c>
       <c r="E40">
-        <v>33.88199059936107</v>
+        <v>33.90415115277162</v>
       </c>
       <c r="G40">
-        <v>34.78829048350811</v>
+        <v>35.08472266995661</v>
       </c>
       <c r="I40">
-        <v>36.12106820859646</v>
+        <v>36.49707992927729</v>
       </c>
       <c r="K40">
-        <v>34.77782585939848</v>
+        <v>35.19329494049256</v>
       </c>
     </row>
   </sheetData>
@@ -3823,7 +3823,7 @@
         <v>113</v>
       </c>
       <c r="G22">
-        <v>29.60157458661558</v>
+        <v>30.37836030090129</v>
       </c>
       <c r="H22">
         <v>200</v>
@@ -3852,7 +3852,7 @@
         <v>113</v>
       </c>
       <c r="G23">
-        <v>15.04636223991063</v>
+        <v>25.43709045963145</v>
       </c>
       <c r="H23">
         <v>200</v>
@@ -3881,7 +3881,7 @@
         <v>113</v>
       </c>
       <c r="G24">
-        <v>13.09814611008896</v>
+        <v>26.27834642448045</v>
       </c>
       <c r="H24">
         <v>200</v>
@@ -3910,7 +3910,7 @@
         <v>113</v>
       </c>
       <c r="G25">
-        <v>10.34287564525967</v>
+        <v>24.9061602772943</v>
       </c>
       <c r="H25">
         <v>200</v>

</xml_diff>